<commit_message>
config from excel returns now all tables from all sheets
</commit_message>
<xml_diff>
--- a/Tests/Test Config From EXCEL/testdata/getattributeasdbl.xlsx
+++ b/Tests/Test Config From EXCEL/testdata/getattributeasdbl.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Rf0d14ad1ada34b7f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R98ad6b9b023e4cf0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -67,7 +67,7 @@
     </x:row>
   </x:sheetData>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raa4497acb85047a8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R89078a83fbbb4d0d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
made json path to excel path sheet or sheetless compatible
</commit_message>
<xml_diff>
--- a/Tests/Test Config From EXCEL/testdata/getattributeasdbl.xlsx
+++ b/Tests/Test Config From EXCEL/testdata/getattributeasdbl.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R98ad6b9b023e4cf0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R45f4cf09f6a74afe"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -67,7 +67,7 @@
     </x:row>
   </x:sheetData>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R89078a83fbbb4d0d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfaa8f8e31c48479a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
adjusted jsonpath to excel and added tests
</commit_message>
<xml_diff>
--- a/Tests/Test Config From EXCEL/testdata/getattributeasdbl.xlsx
+++ b/Tests/Test Config From EXCEL/testdata/getattributeasdbl.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R45f4cf09f6a74afe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Rff524c82a9714268"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -67,7 +67,7 @@
     </x:row>
   </x:sheetData>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfaa8f8e31c48479a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R06ab304b3523466a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
added tests for config from excel
</commit_message>
<xml_diff>
--- a/Tests/Test Config From EXCEL/testdata/getattributeasdbl.xlsx
+++ b/Tests/Test Config From EXCEL/testdata/getattributeasdbl.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Rff524c82a9714268"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R1027db04e61e4708"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -67,7 +67,7 @@
     </x:row>
   </x:sheetData>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R06ab304b3523466a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7a42e09802e848cc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>